<commit_message>
Corrige fundo cinza da coluna F (taxa) nos 5 primeiros bancos da aba INDICES
Na aba INDICES BACARIOS APURAR TX MEDI (Minuta Total), as celulas F7:F11
(posicoes 1 a 5) usavam um estilo com preenchimento cinza claro diferente
do resto da tabela (branco, a partir da posicao 6). Alterado para o mesmo
estilo branco usado nas demais linhas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelos/minuta-total-modelo.xlsx
+++ b/public/modelos/minuta-total-modelo.xlsx
@@ -15542,7 +15542,7 @@
         <v>55</v>
       </c>
       <c r="E7" s="204"/>
-      <c r="F7" s="97">
+      <c r="F7" s="92">
         <v>1.59</v>
       </c>
       <c r="G7" s="92">
@@ -15560,7 +15560,7 @@
         <v>56</v>
       </c>
       <c r="E8" s="204"/>
-      <c r="F8" s="97">
+      <c r="F8" s="92">
         <v>1.64</v>
       </c>
       <c r="G8" s="92">
@@ -15578,7 +15578,7 @@
         <v>57</v>
       </c>
       <c r="E9" s="204"/>
-      <c r="F9" s="97">
+      <c r="F9" s="92">
         <v>1.65</v>
       </c>
       <c r="G9" s="92">
@@ -15597,7 +15597,7 @@
         <v>58</v>
       </c>
       <c r="E10" s="204"/>
-      <c r="F10" s="97">
+      <c r="F10" s="92">
         <v>1.66</v>
       </c>
       <c r="G10" s="92">
@@ -15615,7 +15615,7 @@
         <v>59</v>
       </c>
       <c r="E11" s="204"/>
-      <c r="F11" s="97">
+      <c r="F11" s="92">
         <v>1.69</v>
       </c>
       <c r="G11" s="92">

</xml_diff>